<commit_message>
Atividades desenvolvidas no final de semana dos dias 29 e 30 de novembro (esqueci de commitar por acidente)
</commit_message>
<xml_diff>
--- a/Codigo/resultado_global.xlsx
+++ b/Codigo/resultado_global.xlsx
@@ -703,23 +703,23 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.811708319068812</v>
+        <v>0.8135341777929933</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3779366700715016</v>
+        <v>0.3789581205311542</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6313993174061433</v>
+        <v>0.6396551724137931</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4728434504792332</v>
+        <v>0.4759461193072482</v>
       </c>
       <c r="J6" t="n">
         <v>0.7695074522353704</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[[6373, 432], [1218, 740]]</t>
+          <t>[[6387, 418], [1216, 742]]</t>
         </is>
       </c>
     </row>
@@ -1079,23 +1079,23 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.7940203126783065</v>
+        <v>0.7941344288485679</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3038815117466803</v>
+        <v>0.303370786516854</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5737704918032787</v>
+        <v>0.574468085106383</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3973288814691152</v>
+        <v>0.3970588235294117</v>
       </c>
       <c r="J14" t="n">
         <v>0.7012649924685852</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[[6363, 442], [1363, 595]]</t>
+          <t>[[6365, 440], [1364, 594]]</t>
         </is>
       </c>
     </row>
@@ -1455,23 +1455,23 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.8099965765148922</v>
+        <v>0.8098824603446309</v>
       </c>
       <c r="G22" t="n">
-        <v>0.339632277834525</v>
+        <v>0.3401430030643514</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6412729026036644</v>
+        <v>0.6403846153846153</v>
       </c>
       <c r="I22" t="n">
-        <v>0.4440734557595993</v>
+        <v>0.4442961974649767</v>
       </c>
       <c r="J22" t="n">
         <v>0.7142088937488884</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[[6433, 372], [1293, 665]]</t>
+          <t>[[6431, 374], [1292, 666]]</t>
         </is>
       </c>
     </row>
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.8138765263037773</v>
+        <v>0.8135341777929933</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3621041879468846</v>
       </c>
       <c r="H30" t="n">
-        <v>0.6490428441203282</v>
+        <v>0.6480804387568556</v>
       </c>
       <c r="I30" t="n">
-        <v>0.4661211129296235</v>
+        <v>0.4646133682830931</v>
       </c>
       <c r="J30" t="n">
         <v>0.7691524587986212</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[[6420, 385], [1246, 712]]</t>
+          <t>[[6420, 385], [1249, 709]]</t>
         </is>
       </c>
     </row>
@@ -2207,23 +2207,23 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0.7913956407622961</v>
+        <v>0.7925368024649093</v>
       </c>
       <c r="G38" t="n">
-        <v>0.4274770173646578</v>
+        <v>0.4295199182839632</v>
       </c>
       <c r="H38" t="n">
-        <v>0.542098445595855</v>
+        <v>0.5453955901426718</v>
       </c>
       <c r="I38" t="n">
-        <v>0.4780125642490006</v>
+        <v>0.4805714285714286</v>
       </c>
       <c r="J38" t="n">
         <v>0.754448375473481</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>[[6098, 707], [1121, 837]]</t>
+          <t>[[6104, 701], [1117, 841]]</t>
         </is>
       </c>
     </row>
@@ -2583,23 +2583,23 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>0.7810110692685154</v>
+        <v>0.7806687207577314</v>
       </c>
       <c r="G46" t="n">
-        <v>0.4019407558733402</v>
+        <v>0.3998978549540347</v>
       </c>
       <c r="H46" t="n">
-        <v>0.5127035830618892</v>
+        <v>0.5117647058823529</v>
       </c>
       <c r="I46" t="n">
-        <v>0.4506155167477813</v>
+        <v>0.4489678899082569</v>
       </c>
       <c r="J46" t="n">
         <v>0.7037192504760139</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[[6057, 748], [1171, 787]]</t>
+          <t>[[6058, 747], [1175, 783]]</t>
         </is>
       </c>
     </row>
@@ -2959,23 +2959,23 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.7899121305488987</v>
+        <v>0.7885427365057629</v>
       </c>
       <c r="G54" t="n">
-        <v>0.4126659856996935</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="H54" t="n">
-        <v>0.5390260173448966</v>
+        <v>0.5350701402805611</v>
       </c>
       <c r="I54" t="n">
-        <v>0.4674573329476425</v>
+        <v>0.4636758321273516</v>
       </c>
       <c r="J54" t="n">
         <v>0.6993652146959778</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>[[6114, 691], [1150, 808]]</t>
+          <t>[[6109, 696], [1157, 801]]</t>
         </is>
       </c>
     </row>
@@ -3335,23 +3335,23 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>0.7682300581992468</v>
+        <v>0.7688006390505535</v>
       </c>
       <c r="G62" t="n">
-        <v>0.5097037793667007</v>
+        <v>0.5102145045965271</v>
       </c>
       <c r="H62" t="n">
-        <v>0.4823586273562107</v>
+        <v>0.4835430784123911</v>
       </c>
       <c r="I62" t="n">
-        <v>0.4956543332505587</v>
+        <v>0.496520874751491</v>
       </c>
       <c r="J62" t="n">
         <v>0.7551954002457185</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>[[5734, 1071], [960, 998]]</t>
+          <t>[[5738, 1067], [959, 999]]</t>
         </is>
       </c>
     </row>
@@ -3711,23 +3711,23 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.8142188748145612</v>
+        <v>0.8144471071550838</v>
       </c>
       <c r="G70" t="n">
-        <v>0.36414708886619</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H70" t="n">
-        <v>0.6505474452554745</v>
+        <v>0.652014652014652</v>
       </c>
       <c r="I70" t="n">
-        <v>0.466928618205632</v>
+        <v>0.4668852459016393</v>
       </c>
       <c r="J70" t="n">
         <v>0.7679688596455019</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>[[6422, 383], [1245, 713]]</t>
+          <t>[[6425, 380], [1246, 712]]</t>
         </is>
       </c>
     </row>
@@ -4087,23 +4087,23 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.8004108182129408</v>
+        <v>0.800524934383202</v>
       </c>
       <c r="G78" t="n">
         <v>0.3268641470888662</v>
       </c>
       <c r="H78" t="n">
-        <v>0.5975723622782446</v>
+        <v>0.5981308411214953</v>
       </c>
       <c r="I78" t="n">
-        <v>0.4225817101353582</v>
+        <v>0.4227212681638045</v>
       </c>
       <c r="J78" t="n">
         <v>0.709819883985443</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>[[6374, 431], [1318, 640]]</t>
+          <t>[[6375, 430], [1318, 640]]</t>
         </is>
       </c>
     </row>
@@ -4463,23 +4463,23 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.8087412986420176</v>
+        <v>0.8093118794933242</v>
       </c>
       <c r="G86" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.3212461695607763</v>
       </c>
       <c r="H86" t="n">
-        <v>0.6462655601659751</v>
+        <v>0.6477857878475798</v>
       </c>
       <c r="I86" t="n">
-        <v>0.4264202600958248</v>
+        <v>0.4294981222260157</v>
       </c>
       <c r="J86" t="n">
         <v>0.7134122974829989</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>[[6464, 341], [1335, 623]]</t>
+          <t>[[6463, 342], [1329, 629]]</t>
         </is>
       </c>
     </row>
@@ -4839,23 +4839,23 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0.8145612233253452</v>
+        <v>0.8147894556658678</v>
       </c>
       <c r="G94" t="n">
-        <v>0.4024514811031665</v>
+        <v>0.4034729315628192</v>
       </c>
       <c r="H94" t="n">
-        <v>0.6339501206757844</v>
+        <v>0.6345381526104418</v>
       </c>
       <c r="I94" t="n">
-        <v>0.4923461418306779</v>
+        <v>0.4932875429285045</v>
       </c>
       <c r="J94" t="n">
         <v>0.7698020292415524</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>[[6350, 455], [1170, 788]]</t>
+          <t>[[6350, 455], [1168, 790]]</t>
         </is>
       </c>
     </row>
@@ -5215,23 +5215,23 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.754992582448933</v>
+        <v>0.7554490471299783</v>
       </c>
       <c r="G102" t="n">
         <v>0.5796731358529111</v>
       </c>
       <c r="H102" t="n">
-        <v>0.461569743798292</v>
+        <v>0.4623217922606925</v>
       </c>
       <c r="I102" t="n">
-        <v>0.5139234774733983</v>
+        <v>0.5143893043281215</v>
       </c>
       <c r="J102" t="n">
         <v>0.7422887620185542</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>[[5481, 1324], [823, 1135]]</t>
+          <t>[[5485, 1320], [823, 1135]]</t>
         </is>
       </c>
     </row>
@@ -5591,23 +5591,23 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>0.7798699075659021</v>
+        <v>0.7814675339495607</v>
       </c>
       <c r="G110" t="n">
-        <v>0.4713993871297242</v>
+        <v>0.473953013278856</v>
       </c>
       <c r="H110" t="n">
-        <v>0.5079801871216291</v>
+        <v>0.5118587975730833</v>
       </c>
       <c r="I110" t="n">
-        <v>0.4890066225165563</v>
+        <v>0.4921771413418192</v>
       </c>
       <c r="J110" t="n">
         <v>0.7070209896436482</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>[[5911, 894], [1035, 923]]</t>
+          <t>[[5920, 885], [1030, 928]]</t>
         </is>
       </c>
     </row>
@@ -5967,23 +5967,23 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>0.7912815245920347</v>
+        <v>0.7916238731028187</v>
       </c>
       <c r="G118" t="n">
-        <v>0.4489274770173647</v>
+        <v>0.4468845760980593</v>
       </c>
       <c r="H118" t="n">
-        <v>0.5395948434622467</v>
+        <v>0.5407911001236094</v>
       </c>
       <c r="I118" t="n">
-        <v>0.4901031502648453</v>
+        <v>0.4893736017897092</v>
       </c>
       <c r="J118" t="n">
         <v>0.6778433060471218</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>[[6055, 750], [1079, 879]]</t>
+          <t>[[6062, 743], [1083, 875]]</t>
         </is>
       </c>
     </row>
@@ -6343,23 +6343,23 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0.7475750313819468</v>
+        <v>0.7482597284035147</v>
       </c>
       <c r="G126" t="n">
-        <v>0.5801838610827375</v>
+        <v>0.5786516853932584</v>
       </c>
       <c r="H126" t="n">
-        <v>0.44972288202692</v>
+        <v>0.4506762132060461</v>
       </c>
       <c r="I126" t="n">
-        <v>0.5066904549509367</v>
+        <v>0.5067084078711985</v>
       </c>
       <c r="J126" t="n">
         <v>0.7420519746416105</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>[[5415, 1390], [822, 1136]]</t>
+          <t>[[5424, 1381], [825, 1133]]</t>
         </is>
       </c>
     </row>
@@ -8223,23 +8223,23 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>0.8047856430707876</v>
+        <v>0.8055832502492523</v>
       </c>
       <c r="G166" t="n">
         <v>0.304093567251462</v>
       </c>
       <c r="H166" t="n">
-        <v>0.02749867794817557</v>
+        <v>0.02761550716941051</v>
       </c>
       <c r="I166" t="n">
-        <v>0.0504364694471387</v>
+        <v>0.05063291139240506</v>
       </c>
       <c r="J166" t="n">
         <v>0.6263742749374366</v>
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>[[8020, 1839], [119, 52]]</t>
+          <t>[[8028, 1831], [119, 52]]</t>
         </is>
       </c>
     </row>
@@ -8599,23 +8599,23 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>0.9758723828514456</v>
+        <v>0.9760717846460618</v>
       </c>
       <c r="G174" t="n">
         <v>0.02923976608187134</v>
       </c>
       <c r="H174" t="n">
-        <v>0.06172839506172839</v>
+        <v>0.06329113924050633</v>
       </c>
       <c r="I174" t="n">
-        <v>0.03968253968253968</v>
+        <v>0.04</v>
       </c>
       <c r="J174" t="n">
         <v>0.5560923643252906</v>
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>[[9783, 76], [166, 5]]</t>
+          <t>[[9785, 74], [166, 5]]</t>
         </is>
       </c>
     </row>
@@ -8975,23 +8975,23 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>0.9795613160518445</v>
+        <v>0.9791625124626122</v>
       </c>
       <c r="G182" t="n">
         <v>0.03508771929824561</v>
       </c>
       <c r="H182" t="n">
-        <v>0.1304347826086956</v>
+        <v>0.12</v>
       </c>
       <c r="I182" t="n">
-        <v>0.05529953917050692</v>
+        <v>0.05429864253393665</v>
       </c>
       <c r="J182" t="n">
         <v>0.5427308678092093</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>[[9819, 40], [165, 6]]</t>
+          <t>[[9815, 44], [165, 6]]</t>
         </is>
       </c>
     </row>
@@ -9351,23 +9351,23 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>0.8615154536390828</v>
+        <v>0.8622133599202393</v>
       </c>
       <c r="G190" t="n">
-        <v>0.1929824561403509</v>
+        <v>0.2046783625730994</v>
       </c>
       <c r="H190" t="n">
-        <v>0.02570093457943925</v>
+        <v>0.0273224043715847</v>
       </c>
       <c r="I190" t="n">
-        <v>0.04536082474226804</v>
+        <v>0.04820936639118457</v>
       </c>
       <c r="J190" t="n">
         <v>0.5980076386998195</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>[[8608, 1251], [138, 33]]</t>
+          <t>[[8613, 1246], [136, 35]]</t>
         </is>
       </c>
     </row>
@@ -11231,23 +11231,23 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>0.7616151545363908</v>
+        <v>0.7611166500498504</v>
       </c>
       <c r="G230" t="n">
-        <v>0.3625730994152047</v>
+        <v>0.3801169590643275</v>
       </c>
       <c r="H230" t="n">
-        <v>0.02645051194539249</v>
+        <v>0.02760084925690021</v>
       </c>
       <c r="I230" t="n">
-        <v>0.04930417495029821</v>
+        <v>0.05146476642913698</v>
       </c>
       <c r="J230" t="n">
         <v>0.5579824650377339</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>[[7577, 2282], [109, 62]]</t>
+          <t>[[7569, 2290], [106, 65]]</t>
         </is>
       </c>
     </row>
@@ -11607,23 +11607,23 @@
         </is>
       </c>
       <c r="F238" t="n">
-        <v>0.505284147557328</v>
+        <v>0.5064805583250249</v>
       </c>
       <c r="G238" t="n">
-        <v>0.5672514619883041</v>
+        <v>0.5730994152046783</v>
       </c>
       <c r="H238" t="n">
-        <v>0.01945837512537613</v>
+        <v>0.01969849246231156</v>
       </c>
       <c r="I238" t="n">
-        <v>0.03762606671838634</v>
+        <v>0.038087835211815</v>
       </c>
       <c r="J238" t="n">
         <v>0.5147370319160989</v>
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>[[4971, 4888], [74, 97]]</t>
+          <t>[[4982, 4877], [73, 98]]</t>
         </is>
       </c>
     </row>
@@ -11983,23 +11983,23 @@
         </is>
       </c>
       <c r="F246" t="n">
-        <v>0.5603190428713859</v>
+        <v>0.5612163509471585</v>
       </c>
       <c r="G246" t="n">
-        <v>0.4152046783625731</v>
+        <v>0.4035087719298245</v>
       </c>
       <c r="H246" t="n">
-        <v>0.01620634558320018</v>
+        <v>0.0157967032967033</v>
       </c>
       <c r="I246" t="n">
-        <v>0.03119507908611599</v>
+        <v>0.03040317250495704</v>
       </c>
       <c r="J246" t="n">
         <v>0.4949456933404275</v>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>[[5549, 4310], [100, 71]]</t>
+          <t>[[5560, 4299], [102, 69]]</t>
         </is>
       </c>
     </row>
@@ -12359,23 +12359,23 @@
         </is>
       </c>
       <c r="F254" t="n">
-        <v>0.7756729810568295</v>
+        <v>0.7770687936191426</v>
       </c>
       <c r="G254" t="n">
-        <v>0.3157894736842105</v>
+        <v>0.327485380116959</v>
       </c>
       <c r="H254" t="n">
-        <v>0.02469135802469136</v>
+        <v>0.02572347266881029</v>
       </c>
       <c r="I254" t="n">
-        <v>0.04580152671755725</v>
+        <v>0.04770017035775128</v>
       </c>
       <c r="J254" t="n">
         <v>0.5623172699982028</v>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>[[7726, 2133], [117, 54]]</t>
+          <t>[[7738, 2121], [115, 56]]</t>
         </is>
       </c>
     </row>
@@ -12735,23 +12735,23 @@
         </is>
       </c>
       <c r="F262" t="n">
-        <v>0.9496057593417895</v>
+        <v>0.9499485773054508</v>
       </c>
       <c r="G262" t="n">
-        <v>0.8874734607218684</v>
+        <v>0.89171974522293</v>
       </c>
       <c r="H262" t="n">
-        <v>0.81640625</v>
+        <v>0.8155339805825242</v>
       </c>
       <c r="I262" t="n">
-        <v>0.8504577822990844</v>
+        <v>0.8519269776876268</v>
       </c>
       <c r="J262" t="n">
         <v>0.9823786137252554</v>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>[[2352, 94], [53, 418]]</t>
+          <t>[[2351, 95], [51, 420]]</t>
         </is>
       </c>
     </row>
@@ -13114,20 +13114,20 @@
         <v>0.9019540623928693</v>
       </c>
       <c r="G270" t="n">
-        <v>0.5923566878980892</v>
+        <v>0.5902335456475584</v>
       </c>
       <c r="H270" t="n">
-        <v>0.7479892761394102</v>
+        <v>0.7493261455525606</v>
       </c>
       <c r="I270" t="n">
-        <v>0.6611374407582938</v>
+        <v>0.6603325415676959</v>
       </c>
       <c r="J270" t="n">
         <v>0.9193405586138294</v>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>[[2352, 94], [192, 279]]</t>
+          <t>[[2353, 93], [193, 278]]</t>
         </is>
       </c>
     </row>
@@ -13487,23 +13487,23 @@
         </is>
       </c>
       <c r="F278" t="n">
-        <v>0.9019540623928693</v>
+        <v>0.901611244429208</v>
       </c>
       <c r="G278" t="n">
-        <v>0.5583864118895966</v>
+        <v>0.5520169851380042</v>
       </c>
       <c r="H278" t="n">
-        <v>0.7712609970674487</v>
+        <v>0.7738095238095238</v>
       </c>
       <c r="I278" t="n">
-        <v>0.6477832512315271</v>
+        <v>0.644361833952912</v>
       </c>
       <c r="J278" t="n">
         <v>0.9246657743566775</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>[[2368, 78], [208, 263]]</t>
+          <t>[[2370, 76], [211, 260]]</t>
         </is>
       </c>
     </row>
@@ -13863,23 +13863,23 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>0.9595474802879671</v>
+        <v>0.9602331162152897</v>
       </c>
       <c r="G286" t="n">
-        <v>0.8365180467091295</v>
+        <v>0.8428874734607219</v>
       </c>
       <c r="H286" t="n">
-        <v>0.9057471264367816</v>
+        <v>0.9043280182232346</v>
       </c>
       <c r="I286" t="n">
-        <v>0.869757174392936</v>
+        <v>0.8725274725274725</v>
       </c>
       <c r="J286" t="n">
         <v>0.9898052715729828</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>[[2405, 41], [77, 394]]</t>
+          <t>[[2404, 42], [74, 397]]</t>
         </is>
       </c>
     </row>
@@ -14239,23 +14239,23 @@
         </is>
       </c>
       <c r="F294" t="n">
-        <v>0.826191292423723</v>
+        <v>0.816935207404868</v>
       </c>
       <c r="G294" t="n">
         <v>0.881104033970276</v>
       </c>
       <c r="H294" t="n">
-        <v>0.4792147806004619</v>
+        <v>0.4647256438969765</v>
       </c>
       <c r="I294" t="n">
-        <v>0.6207928197456993</v>
+        <v>0.6085043988269795</v>
       </c>
       <c r="J294" t="n">
         <v>0.9764397178633863</v>
       </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>[[1995, 451], [56, 415]]</t>
+          <t>[[1968, 478], [56, 415]]</t>
         </is>
       </c>
     </row>
@@ -14615,23 +14615,23 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>0.8333904696606103</v>
+        <v>0.8368186492972232</v>
       </c>
       <c r="G302" t="n">
-        <v>0.7685774946921444</v>
+        <v>0.7664543524416136</v>
       </c>
       <c r="H302" t="n">
-        <v>0.489851150202977</v>
+        <v>0.4965612104539202</v>
       </c>
       <c r="I302" t="n">
-        <v>0.5983471074380166</v>
+        <v>0.6026711185308848</v>
       </c>
       <c r="J302" t="n">
         <v>0.9004978881418253</v>
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>[[2069, 377], [109, 362]]</t>
+          <t>[[2080, 366], [110, 361]]</t>
         </is>
       </c>
     </row>
@@ -14991,23 +14991,23 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>0.8488172780253685</v>
+        <v>0.8467603702434008</v>
       </c>
       <c r="G310" t="n">
-        <v>0.7834394904458599</v>
+        <v>0.7813163481953291</v>
       </c>
       <c r="H310" t="n">
-        <v>0.5211864406779662</v>
+        <v>0.5168539325842697</v>
       </c>
       <c r="I310" t="n">
-        <v>0.6259541984732825</v>
+        <v>0.6221470836855453</v>
       </c>
       <c r="J310" t="n">
         <v>0.9092057225888099</v>
       </c>
       <c r="K310" t="inlineStr">
         <is>
-          <t>[[2107, 339], [102, 369]]</t>
+          <t>[[2102, 344], [103, 368]]</t>
         </is>
       </c>
     </row>
@@ -15367,23 +15367,23 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>0.8268769283510456</v>
+        <v>0.8426465546794653</v>
       </c>
       <c r="G318" t="n">
         <v>0.881104033970276</v>
       </c>
       <c r="H318" t="n">
-        <v>0.4803240740740741</v>
+        <v>0.5073349633251834</v>
       </c>
       <c r="I318" t="n">
-        <v>0.6217228464419475</v>
+        <v>0.6439100077579519</v>
       </c>
       <c r="J318" t="n">
         <v>0.9875467204135874</v>
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>[[1997, 449], [56, 415]]</t>
+          <t>[[2043, 403], [56, 415]]</t>
         </is>
       </c>
     </row>
@@ -16119,23 +16119,23 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>0.9070963318477888</v>
+        <v>0.9067535138841275</v>
       </c>
       <c r="G334" t="n">
         <v>0.6050955414012739</v>
       </c>
       <c r="H334" t="n">
-        <v>0.7702702702702703</v>
+        <v>0.7681940700808625</v>
       </c>
       <c r="I334" t="n">
-        <v>0.6777645659928656</v>
+        <v>0.6769596199524941</v>
       </c>
       <c r="J334" t="n">
         <v>0.9146837073570439</v>
       </c>
       <c r="K334" t="inlineStr">
         <is>
-          <t>[[2361, 85], [186, 285]]</t>
+          <t>[[2360, 86], [186, 285]]</t>
         </is>
       </c>
     </row>
@@ -16495,23 +16495,23 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>0.9053822420294824</v>
+        <v>0.9043537881384984</v>
       </c>
       <c r="G342" t="n">
-        <v>0.6921443736730361</v>
+        <v>0.6900212314225053</v>
       </c>
       <c r="H342" t="n">
-        <v>0.7133479212253829</v>
+        <v>0.7096069868995634</v>
       </c>
       <c r="I342" t="n">
-        <v>0.7025862068965517</v>
+        <v>0.6996770721205597</v>
       </c>
       <c r="J342" t="n">
         <v>0.9238420368277512</v>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>[[2315, 131], [145, 326]]</t>
+          <t>[[2313, 133], [146, 325]]</t>
         </is>
       </c>
     </row>
@@ -16871,23 +16871,23 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>0.9681179293794995</v>
+        <v>0.9698320191978059</v>
       </c>
       <c r="G350" t="n">
-        <v>0.8662420382165605</v>
+        <v>0.8726114649681529</v>
       </c>
       <c r="H350" t="n">
-        <v>0.9315068493150684</v>
+        <v>0.9362186788154897</v>
       </c>
       <c r="I350" t="n">
-        <v>0.8976897689768977</v>
+        <v>0.9032967032967033</v>
       </c>
       <c r="J350" t="n">
         <v>0.9906368211543436</v>
       </c>
       <c r="K350" t="inlineStr">
         <is>
-          <t>[[2416, 30], [63, 408]]</t>
+          <t>[[2418, 28], [60, 411]]</t>
         </is>
       </c>
     </row>
@@ -17247,23 +17247,23 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>0.9369214946863216</v>
+        <v>0.9372643126499829</v>
       </c>
       <c r="G358" t="n">
         <v>0.8535031847133758</v>
       </c>
       <c r="H358" t="n">
-        <v>0.7775628626692457</v>
+        <v>0.7790697674418605</v>
       </c>
       <c r="I358" t="n">
-        <v>0.8137651821862348</v>
+        <v>0.8145896656534954</v>
       </c>
       <c r="J358" t="n">
         <v>0.9796001270760529</v>
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>[[2331, 115], [69, 402]]</t>
+          <t>[[2332, 114], [69, 402]]</t>
         </is>
       </c>
     </row>
@@ -17623,23 +17623,23 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>0.8560164552622558</v>
+        <v>0.8577305450805622</v>
       </c>
       <c r="G366" t="n">
-        <v>0.8259023354564756</v>
+        <v>0.8301486199575372</v>
       </c>
       <c r="H366" t="n">
-        <v>0.5350756533700137</v>
+        <v>0.5385674931129476</v>
       </c>
       <c r="I366" t="n">
-        <v>0.6494156928213689</v>
+        <v>0.6532999164578112</v>
       </c>
       <c r="J366" t="n">
         <v>0.9155656012763157</v>
       </c>
       <c r="K366" t="inlineStr">
         <is>
-          <t>[[2108, 338], [82, 389]]</t>
+          <t>[[2111, 335], [80, 391]]</t>
         </is>
       </c>
     </row>
@@ -17999,23 +17999,23 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>0.8464175522797395</v>
+        <v>0.8467603702434008</v>
       </c>
       <c r="G374" t="n">
         <v>0.8407643312101911</v>
       </c>
       <c r="H374" t="n">
-        <v>0.5149544863459038</v>
+        <v>0.515625</v>
       </c>
       <c r="I374" t="n">
-        <v>0.6387096774193548</v>
+        <v>0.639225181598063</v>
       </c>
       <c r="J374" t="n">
         <v>0.9200740235368461</v>
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>[[2073, 373], [75, 396]]</t>
+          <t>[[2074, 372], [75, 396]]</t>
         </is>
       </c>
     </row>
@@ -18375,23 +18375,23 @@
         </is>
       </c>
       <c r="F382" t="n">
-        <v>0.9499485773054508</v>
+        <v>0.9526911210147412</v>
       </c>
       <c r="G382" t="n">
         <v>0.8747346072186837</v>
       </c>
       <c r="H382" t="n">
-        <v>0.8256513026052105</v>
+        <v>0.8391038696537678</v>
       </c>
       <c r="I382" t="n">
-        <v>0.8494845360824742</v>
+        <v>0.8565488565488566</v>
       </c>
       <c r="J382" t="n">
         <v>0.9870424090286495</v>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>[[2359, 87], [59, 412]]</t>
+          <t>[[2367, 79], [59, 412]]</t>
         </is>
       </c>
     </row>
@@ -18751,23 +18751,23 @@
         </is>
       </c>
       <c r="F390" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7456445993031359</v>
       </c>
       <c r="G390" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5747126436781609</v>
       </c>
       <c r="H390" t="n">
-        <v>0.5581395348837209</v>
+        <v>0.5813953488372093</v>
       </c>
       <c r="I390" t="n">
-        <v>0.5549132947976878</v>
+        <v>0.5780346820809249</v>
       </c>
       <c r="J390" t="n">
         <v>0.7898275862068965</v>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>[[162, 38], [39, 48]]</t>
+          <t>[[164, 36], [37, 50]]</t>
         </is>
       </c>
     </row>
@@ -19130,20 +19130,20 @@
         <v>0.7630662020905923</v>
       </c>
       <c r="G398" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4022988505747127</v>
       </c>
       <c r="H398" t="n">
-        <v>0.6938775510204082</v>
+        <v>0.6862745098039216</v>
       </c>
       <c r="I398" t="n">
-        <v>0.5</v>
+        <v>0.5072463768115942</v>
       </c>
       <c r="J398" t="n">
         <v>0.7922988505747127</v>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t>[[185, 15], [53, 34]]</t>
+          <t>[[184, 16], [52, 35]]</t>
         </is>
       </c>
     </row>
@@ -19503,23 +19503,23 @@
         </is>
       </c>
       <c r="F406" t="n">
-        <v>0.7735191637630662</v>
+        <v>0.7770034843205574</v>
       </c>
       <c r="G406" t="n">
         <v>0.4137931034482759</v>
       </c>
       <c r="H406" t="n">
-        <v>0.72</v>
+        <v>0.7346938775510204</v>
       </c>
       <c r="I406" t="n">
-        <v>0.5255474452554745</v>
+        <v>0.5294117647058824</v>
       </c>
       <c r="J406" t="n">
         <v>0.8070114942528736</v>
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t>[[186, 14], [51, 36]]</t>
+          <t>[[187, 13], [51, 36]]</t>
         </is>
       </c>
     </row>
@@ -19879,23 +19879,23 @@
         </is>
       </c>
       <c r="F414" t="n">
-        <v>0.7456445993031359</v>
+        <v>0.7665505226480837</v>
       </c>
       <c r="G414" t="n">
         <v>0.4597701149425287</v>
       </c>
       <c r="H414" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I414" t="n">
-        <v>0.5228758169934641</v>
+        <v>0.54421768707483</v>
       </c>
       <c r="J414" t="n">
         <v>0.7791954022988505</v>
       </c>
       <c r="K414" t="inlineStr">
         <is>
-          <t>[[174, 26], [47, 40]]</t>
+          <t>[[180, 20], [47, 40]]</t>
         </is>
       </c>
     </row>
@@ -20258,20 +20258,20 @@
         <v>0.7421602787456446</v>
       </c>
       <c r="G422" t="n">
-        <v>0.3563218390804598</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="H422" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6274509803921569</v>
       </c>
       <c r="I422" t="n">
-        <v>0.4558823529411765</v>
+        <v>0.463768115942029</v>
       </c>
       <c r="J422" t="n">
         <v>0.7988505747126438</v>
       </c>
       <c r="K422" t="inlineStr">
         <is>
-          <t>[[182, 18], [56, 31]]</t>
+          <t>[[181, 19], [55, 32]]</t>
         </is>
       </c>
     </row>
@@ -20631,23 +20631,23 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>0.7804878048780488</v>
+        <v>0.7770034843205574</v>
       </c>
       <c r="G430" t="n">
         <v>0.5287356321839081</v>
       </c>
       <c r="H430" t="n">
-        <v>0.6764705882352942</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I430" t="n">
-        <v>0.5935483870967742</v>
+        <v>0.5897435897435898</v>
       </c>
       <c r="J430" t="n">
         <v>0.7986206896551725</v>
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t>[[178, 22], [41, 46]]</t>
+          <t>[[177, 23], [41, 46]]</t>
         </is>
       </c>
     </row>
@@ -21007,23 +21007,23 @@
         </is>
       </c>
       <c r="F438" t="n">
-        <v>0.7665505226480837</v>
+        <v>0.7630662020905923</v>
       </c>
       <c r="G438" t="n">
-        <v>0.5977011494252874</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="H438" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.6144578313253012</v>
       </c>
       <c r="I438" t="n">
-        <v>0.6081871345029239</v>
+        <v>0.6</v>
       </c>
       <c r="J438" t="n">
         <v>0.8017816091954024</v>
       </c>
       <c r="K438" t="inlineStr">
         <is>
-          <t>[[168, 32], [35, 52]]</t>
+          <t>[[168, 32], [36, 51]]</t>
         </is>
       </c>
     </row>
@@ -21383,23 +21383,23 @@
         </is>
       </c>
       <c r="F446" t="n">
-        <v>0.7630662020905923</v>
+        <v>0.7560975609756098</v>
       </c>
       <c r="G446" t="n">
-        <v>0.5172413793103449</v>
+        <v>0.5287356321839081</v>
       </c>
       <c r="H446" t="n">
-        <v>0.6338028169014085</v>
+        <v>0.6133333333333333</v>
       </c>
       <c r="I446" t="n">
-        <v>0.569620253164557</v>
+        <v>0.5679012345679012</v>
       </c>
       <c r="J446" t="n">
         <v>0.7943678160919538</v>
       </c>
       <c r="K446" t="inlineStr">
         <is>
-          <t>[[174, 26], [42, 45]]</t>
+          <t>[[171, 29], [41, 46]]</t>
         </is>
       </c>
     </row>
@@ -21759,23 +21759,23 @@
         </is>
       </c>
       <c r="F454" t="n">
-        <v>0.7456445993031359</v>
+        <v>0.7665505226480837</v>
       </c>
       <c r="G454" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5632183908045977</v>
       </c>
       <c r="H454" t="n">
-        <v>0.5853658536585366</v>
+        <v>0.6282051282051282</v>
       </c>
       <c r="I454" t="n">
-        <v>0.5680473372781065</v>
+        <v>0.593939393939394</v>
       </c>
       <c r="J454" t="n">
         <v>0.7969540229885058</v>
       </c>
       <c r="K454" t="inlineStr">
         <is>
-          <t>[[166, 34], [39, 48]]</t>
+          <t>[[171, 29], [38, 49]]</t>
         </is>
       </c>
     </row>
@@ -22511,23 +22511,23 @@
         </is>
       </c>
       <c r="F470" t="n">
-        <v>0.7630662020905923</v>
+        <v>0.7526132404181185</v>
       </c>
       <c r="G470" t="n">
-        <v>0.6091954022988506</v>
+        <v>0.5747126436781609</v>
       </c>
       <c r="H470" t="n">
-        <v>0.6091954022988506</v>
+        <v>0.5952380952380952</v>
       </c>
       <c r="I470" t="n">
-        <v>0.6091954022988506</v>
+        <v>0.5847953216374269</v>
       </c>
       <c r="J470" t="n">
         <v>0.8052873563218391</v>
       </c>
       <c r="K470" t="inlineStr">
         <is>
-          <t>[[166, 34], [34, 53]]</t>
+          <t>[[166, 34], [37, 50]]</t>
         </is>
       </c>
     </row>
@@ -23263,23 +23263,23 @@
         </is>
       </c>
       <c r="F486" t="n">
-        <v>0.735191637630662</v>
+        <v>0.7386759581881533</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3563218390804598</v>
+        <v>0.4022988505747127</v>
       </c>
       <c r="H486" t="n">
-        <v>0.6078431372549019</v>
+        <v>0.603448275862069</v>
       </c>
       <c r="I486" t="n">
-        <v>0.4492753623188406</v>
+        <v>0.4827586206896552</v>
       </c>
       <c r="J486" t="n">
         <v>0.7755172413793102</v>
       </c>
       <c r="K486" t="inlineStr">
         <is>
-          <t>[[180, 20], [56, 31]]</t>
+          <t>[[177, 23], [52, 35]]</t>
         </is>
       </c>
     </row>
@@ -23639,23 +23639,23 @@
         </is>
       </c>
       <c r="F494" t="n">
-        <v>0.7282229965156795</v>
+        <v>0.7456445993031359</v>
       </c>
       <c r="G494" t="n">
-        <v>0.4712643678160919</v>
+        <v>0.4942528735632184</v>
       </c>
       <c r="H494" t="n">
-        <v>0.5616438356164384</v>
+        <v>0.5972222222222222</v>
       </c>
       <c r="I494" t="n">
-        <v>0.5125</v>
+        <v>0.5408805031446541</v>
       </c>
       <c r="J494" t="n">
         <v>0.7848850574712642</v>
       </c>
       <c r="K494" t="inlineStr">
         <is>
-          <t>[[168, 32], [46, 41]]</t>
+          <t>[[171, 29], [44, 43]]</t>
         </is>
       </c>
     </row>
@@ -24015,23 +24015,23 @@
         </is>
       </c>
       <c r="F502" t="n">
-        <v>0.7456445993031359</v>
+        <v>0.7421602787456446</v>
       </c>
       <c r="G502" t="n">
-        <v>0.6551724137931034</v>
+        <v>0.632183908045977</v>
       </c>
       <c r="H502" t="n">
-        <v>0.57</v>
+        <v>0.5670103092783505</v>
       </c>
       <c r="I502" t="n">
-        <v>0.6096256684491979</v>
+        <v>0.5978260869565217</v>
       </c>
       <c r="J502" t="n">
         <v>0.7827011494252873</v>
       </c>
       <c r="K502" t="inlineStr">
         <is>
-          <t>[[157, 43], [30, 57]]</t>
+          <t>[[158, 42], [32, 55]]</t>
         </is>
       </c>
     </row>
@@ -24394,20 +24394,20 @@
         <v>0.7386759581881533</v>
       </c>
       <c r="G510" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="H510" t="n">
-        <v>0.6111111111111112</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="I510" t="n">
-        <v>0.4680851063829787</v>
+        <v>0.460431654676259</v>
       </c>
       <c r="J510" t="n">
         <v>0.7617816091954023</v>
       </c>
       <c r="K510" t="inlineStr">
         <is>
-          <t>[[179, 21], [54, 33]]</t>
+          <t>[[180, 20], [55, 32]]</t>
         </is>
       </c>
     </row>
@@ -24860,22 +24860,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.001184804663860839</v>
+        <v>-0.0005782727394705867</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06134412714601389</v>
+        <v>0.06314592894781573</v>
       </c>
       <c r="I6" t="n">
-        <v>0.06134412714601389</v>
+        <v>0.06314592894781573</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0001043620581853005</v>
+        <v>-0.002780536246276069</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.06134412714601389</v>
+        <v>-0.06314592894781579</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.01562097358055292</v>
+        <v>-0.004477458152626901</v>
       </c>
     </row>
     <row r="7">
@@ -25254,22 +25254,22 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>-0.005332223411858447</v>
+        <v>-0.003973318071913062</v>
       </c>
       <c r="H14" t="n">
-        <v>0.03680095189529153</v>
+        <v>0.04006034336223013</v>
       </c>
       <c r="I14" t="n">
-        <v>0.03680095189529153</v>
+        <v>0.04006034336223013</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.005254422744492254</v>
+        <v>-0.004474695648975693</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.03680095189529164</v>
+        <v>-0.04006034336223019</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.007573703172819912</v>
+        <v>-0.00764685436218282</v>
       </c>
     </row>
     <row r="15">
@@ -25654,22 +25654,22 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.002826301853002949</v>
+        <v>0.003387049516554344</v>
       </c>
       <c r="H22" t="n">
-        <v>0.06034123746387898</v>
+        <v>0.06124213836477987</v>
       </c>
       <c r="I22" t="n">
-        <v>0.06034123746387898</v>
+        <v>0.06124213836477987</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0007617970502776863</v>
+        <v>0.001233495163485233</v>
       </c>
       <c r="K22" t="n">
-        <v>-0.06034123746387898</v>
+        <v>-0.06124213836477987</v>
       </c>
       <c r="L22" t="n">
-        <v>-0.01538600671589563</v>
+        <v>-0.01679738255138619</v>
       </c>
     </row>
     <row r="23">
@@ -26054,22 +26054,22 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.002043423852175999</v>
+        <v>0.003882242442995565</v>
       </c>
       <c r="H30" t="n">
-        <v>0.05692036375998638</v>
+        <v>0.0625382457929628</v>
       </c>
       <c r="I30" t="n">
-        <v>0.05692036375998638</v>
+        <v>0.0625382457929628</v>
       </c>
       <c r="J30" t="n">
-        <v>0.001950696973040567</v>
+        <v>0.002576409577402627</v>
       </c>
       <c r="K30" t="n">
-        <v>-0.05692036375998644</v>
+        <v>-0.06253824579296285</v>
       </c>
       <c r="L30" t="n">
-        <v>-0.02483672510189328</v>
+        <v>-0.02362617139945067</v>
       </c>
     </row>
     <row r="31">
@@ -26454,22 +26454,22 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0.09855248349493825</v>
+        <v>0.1000983047227341</v>
       </c>
       <c r="H38" t="n">
-        <v>0.2485785313615502</v>
+        <v>0.2459416964133945</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2485785313615502</v>
+        <v>0.2459416964133945</v>
       </c>
       <c r="J38" t="n">
-        <v>0.07101125455147303</v>
+        <v>0.0739761484423848</v>
       </c>
       <c r="K38" t="n">
-        <v>-0.2485785313615502</v>
+        <v>-0.2459416964133945</v>
       </c>
       <c r="L38" t="n">
-        <v>-0.09621476084890723</v>
+        <v>-0.1101597160603371</v>
       </c>
     </row>
     <row r="39">
@@ -26854,22 +26854,22 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0.07479423096407087</v>
+        <v>0.07577930452831533</v>
       </c>
       <c r="H46" t="n">
-        <v>0.1473695393506714</v>
+        <v>0.1520865204827469</v>
       </c>
       <c r="I46" t="n">
-        <v>0.1473695393506714</v>
+        <v>0.1520865204827469</v>
       </c>
       <c r="J46" t="n">
-        <v>0.06879252638934863</v>
+        <v>0.06855667733274487</v>
       </c>
       <c r="K46" t="n">
-        <v>-0.1473695393506714</v>
+        <v>-0.152086520482747</v>
       </c>
       <c r="L46" t="n">
-        <v>-0.1378496644628716</v>
+        <v>-0.133862712629836</v>
       </c>
     </row>
     <row r="47">
@@ -27254,22 +27254,22 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>0.07286439151019605</v>
+        <v>0.07249055973449511</v>
       </c>
       <c r="H54" t="n">
-        <v>0.1579678735339113</v>
+        <v>0.1641424443311236</v>
       </c>
       <c r="I54" t="n">
-        <v>0.1579678735339113</v>
+        <v>0.1641424443311236</v>
       </c>
       <c r="J54" t="n">
-        <v>0.06410910662400238</v>
+        <v>0.06153407628084888</v>
       </c>
       <c r="K54" t="n">
-        <v>-0.1579678735339112</v>
+        <v>-0.1641424443311236</v>
       </c>
       <c r="L54" t="n">
-        <v>-0.1337906556978722</v>
+        <v>-0.1199008868022953</v>
       </c>
     </row>
     <row r="55">
@@ -27654,22 +27654,22 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>0.1294954694940456</v>
+        <v>0.12845480857962</v>
       </c>
       <c r="H62" t="n">
-        <v>0.2147310045894951</v>
+        <v>0.2114716131225565</v>
       </c>
       <c r="I62" t="n">
-        <v>0.2147310045894951</v>
+        <v>0.2114716131225565</v>
       </c>
       <c r="J62" t="n">
-        <v>0.1230718305196955</v>
+        <v>0.1227541468976424</v>
       </c>
       <c r="K62" t="n">
-        <v>-0.2147310045894951</v>
+        <v>-0.2114716131225565</v>
       </c>
       <c r="L62" t="n">
-        <v>-0.1774067529281187</v>
+        <v>-0.1795004829046869</v>
       </c>
     </row>
     <row r="63">
@@ -28054,22 +28054,22 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>0.01062726645486345</v>
+        <v>0.01233111902698887</v>
       </c>
       <c r="H70" t="n">
-        <v>0.03373940442905959</v>
+        <v>0.03673279190520568</v>
       </c>
       <c r="I70" t="n">
-        <v>0.03373940442905959</v>
+        <v>0.03673279190520568</v>
       </c>
       <c r="J70" t="n">
-        <v>0.001854007183919211</v>
+        <v>0.003184564827966863</v>
       </c>
       <c r="K70" t="n">
-        <v>-0.03373940442905954</v>
+        <v>-0.03673279190520573</v>
       </c>
       <c r="L70" t="n">
-        <v>0.02014805503177597</v>
+        <v>0.01658249158249159</v>
       </c>
     </row>
     <row r="71">
@@ -28450,22 +28450,22 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>0.006873743086978371</v>
+        <v>0.006567370537958764</v>
       </c>
       <c r="H78" t="n">
-        <v>0.00701613031598361</v>
+        <v>0.006619933802512926</v>
       </c>
       <c r="I78" t="n">
         <v>0.0002618381928726765</v>
       </c>
       <c r="J78" t="n">
-        <v>0.00701613031598361</v>
+        <v>0.006619933802512926</v>
       </c>
       <c r="K78" t="n">
         <v>-0.000261838192872732</v>
       </c>
       <c r="L78" t="n">
-        <v>-0.01890680541960743</v>
+        <v>-0.01748458110779949</v>
       </c>
     </row>
     <row r="79">
@@ -28850,22 +28850,22 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>0.01022044114972775</v>
+        <v>0.009435706224661167</v>
       </c>
       <c r="H86" t="n">
-        <v>0.0250809923223716</v>
+        <v>0.02232725336173613</v>
       </c>
       <c r="I86" t="n">
-        <v>0.0250809923223716</v>
+        <v>0.02232725336173613</v>
       </c>
       <c r="J86" t="n">
-        <v>0.004107357501598297</v>
+        <v>0.003873767218954056</v>
       </c>
       <c r="K86" t="n">
-        <v>-0.0250809923223716</v>
+        <v>-0.02232725336173613</v>
       </c>
       <c r="L86" t="n">
-        <v>0.006164383561643838</v>
+        <v>0.005155923306196852</v>
       </c>
     </row>
     <row r="87">
@@ -29250,22 +29250,22 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>0.01318856102179006</v>
+        <v>0.01380130611982927</v>
       </c>
       <c r="H94" t="n">
-        <v>0.0308170239204722</v>
+        <v>0.03134735720942616</v>
       </c>
       <c r="I94" t="n">
-        <v>0.0308170239204722</v>
+        <v>0.03134735720942616</v>
       </c>
       <c r="J94" t="n">
-        <v>0.005818471105326253</v>
+        <v>0.006448257901441184</v>
       </c>
       <c r="K94" t="n">
-        <v>-0.03081702392047225</v>
+        <v>-0.03134735720942616</v>
       </c>
       <c r="L94" t="n">
-        <v>0.004596579667723644</v>
+        <v>0.00271272633045061</v>
       </c>
     </row>
     <row r="95">
@@ -29650,22 +29650,22 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>0.1445550260475167</v>
+        <v>0.1447942072355402</v>
       </c>
       <c r="H102" t="n">
-        <v>0.1499844672258466</v>
+        <v>0.1478120978120978</v>
       </c>
       <c r="I102" t="n">
-        <v>0.1499844672258466</v>
+        <v>0.1478120978120978</v>
       </c>
       <c r="J102" t="n">
-        <v>0.140394238205079</v>
+        <v>0.1413285993356559</v>
       </c>
       <c r="K102" t="n">
-        <v>-0.1499844672258466</v>
+        <v>-0.1478120978120978</v>
       </c>
       <c r="L102" t="n">
-        <v>-0.09993489324874755</v>
+        <v>-0.1024571120569485</v>
       </c>
     </row>
     <row r="103">
@@ -30050,22 +30050,22 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>0.09530743557652194</v>
+        <v>0.09603484055924605</v>
       </c>
       <c r="H110" t="n">
-        <v>0.1372165268716993</v>
+        <v>0.1331114365597124</v>
       </c>
       <c r="I110" t="n">
-        <v>0.1372165268716993</v>
+        <v>0.1331114365597124</v>
       </c>
       <c r="J110" t="n">
-        <v>0.08087221352891245</v>
+        <v>0.08297452607271064</v>
       </c>
       <c r="K110" t="n">
-        <v>-0.1372165268716993</v>
+        <v>-0.1331114365597125</v>
       </c>
       <c r="L110" t="n">
-        <v>-0.06826367652055726</v>
+        <v>-0.07587575193284518</v>
       </c>
     </row>
     <row r="111">
@@ -30450,22 +30450,22 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>0.1104547417712311</v>
+        <v>0.1070846437320154</v>
       </c>
       <c r="H118" t="n">
-        <v>0.1559623663071938</v>
+        <v>0.1549016997292859</v>
       </c>
       <c r="I118" t="n">
-        <v>0.1559623663071938</v>
+        <v>0.1549016997292859</v>
       </c>
       <c r="J118" t="n">
-        <v>0.09498582355012067</v>
+        <v>0.09095287436359603</v>
       </c>
       <c r="K118" t="n">
-        <v>-0.1559623663071938</v>
+        <v>-0.1549016997292859</v>
       </c>
       <c r="L118" t="n">
-        <v>-0.1117396707426689</v>
+        <v>-0.1051700106371272</v>
       </c>
     </row>
     <row r="119">
@@ -30850,22 +30850,22 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>0.1694760009841361</v>
+        <v>0.1653113066012002</v>
       </c>
       <c r="H126" t="n">
-        <v>0.1904384680246749</v>
+        <v>0.1863844139706209</v>
       </c>
       <c r="I126" t="n">
-        <v>0.1904384680246749</v>
+        <v>0.1863844139706209</v>
       </c>
       <c r="J126" t="n">
-        <v>0.1608751269291096</v>
+        <v>0.1566795715117585</v>
       </c>
       <c r="K126" t="n">
-        <v>-0.1904384680246749</v>
+        <v>-0.1863844139706209</v>
       </c>
       <c r="L126" t="n">
-        <v>-0.09860248447204967</v>
+        <v>-0.09645919384703033</v>
       </c>
     </row>
     <row r="127">
@@ -32794,7 +32794,7 @@
         </is>
       </c>
       <c r="G166" t="n">
-        <v>0.2567985773814263</v>
+        <v>0.2555882899381586</v>
       </c>
       <c r="H166" t="n">
         <v>0.4053030303030303</v>
@@ -32803,13 +32803,13 @@
         <v>0.4053030303030303</v>
       </c>
       <c r="J166" t="n">
-        <v>0.2548564996246587</v>
+        <v>0.2536278097152746</v>
       </c>
       <c r="K166" t="n">
         <v>-0.4053030303030303</v>
       </c>
       <c r="L166" t="n">
-        <v>-0.05000415110004151</v>
+        <v>-0.04989076232884709</v>
       </c>
     </row>
     <row r="167">
@@ -33188,7 +33188,7 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>0.00870469163326875</v>
+        <v>0.008402119772451807</v>
       </c>
       <c r="H174" t="n">
         <v>0.04545454545454545</v>
@@ -33197,13 +33197,13 @@
         <v>-0.04545454545454545</v>
       </c>
       <c r="J174" t="n">
-        <v>0.009863466054230071</v>
+        <v>0.009556293576884043</v>
       </c>
       <c r="K174" t="n">
         <v>0.04545454545454553</v>
       </c>
       <c r="L174" t="n">
-        <v>-0.4863013698630137</v>
+        <v>-0.4859154929577465</v>
       </c>
     </row>
     <row r="175">
@@ -33588,7 +33588,7 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>0.005184418433880971</v>
+        <v>0.00578956215551486</v>
       </c>
       <c r="H182" t="n">
         <v>0.03535353535353535</v>
@@ -33597,13 +33597,13 @@
         <v>-0.03535353535353535</v>
       </c>
       <c r="J182" t="n">
-        <v>0.006143449546920596</v>
+        <v>0.006757794501612655</v>
       </c>
       <c r="K182" t="n">
         <v>0.03535353535353536</v>
       </c>
       <c r="L182" t="n">
-        <v>-0.9523809523809523</v>
+        <v>-0.9565217391304348</v>
       </c>
     </row>
     <row r="183">
@@ -33984,22 +33984,22 @@
         </is>
       </c>
       <c r="G190" t="n">
-        <v>0.1840464120462528</v>
+        <v>0.1835925542550274</v>
       </c>
       <c r="H190" t="n">
-        <v>0.2613636363636364</v>
+        <v>0.2815656565656566</v>
       </c>
       <c r="I190" t="n">
-        <v>0.2613636363636364</v>
+        <v>0.2815656565656566</v>
       </c>
       <c r="J190" t="n">
-        <v>0.1830909441553464</v>
+        <v>0.1823230129619813</v>
       </c>
       <c r="K190" t="n">
-        <v>-0.2613636363636364</v>
+        <v>-0.2815656565656567</v>
       </c>
       <c r="L190" t="n">
-        <v>-0.1066441402613523</v>
+        <v>-0.1049975807009055</v>
       </c>
     </row>
     <row r="191">
@@ -35922,22 +35922,22 @@
         </is>
       </c>
       <c r="G230" t="n">
-        <v>0.3603533563210982</v>
+        <v>0.367386367803498</v>
       </c>
       <c r="H230" t="n">
-        <v>0.3603606215882468</v>
+        <v>0.4116579265832997</v>
       </c>
       <c r="I230" t="n">
-        <v>0.3305768455022186</v>
+        <v>0.4116579265832997</v>
       </c>
       <c r="J230" t="n">
-        <v>0.3603606215882468</v>
+        <v>0.3657804042747175</v>
       </c>
       <c r="K230" t="n">
-        <v>-0.3305768455022186</v>
+        <v>-0.4116579265832997</v>
       </c>
       <c r="L230" t="n">
-        <v>-0.002526717714395506</v>
+        <v>0.0003426978986216765</v>
       </c>
     </row>
     <row r="231">
@@ -36318,22 +36318,22 @@
         </is>
       </c>
       <c r="G238" t="n">
-        <v>0.1303993559277208</v>
+        <v>0.1260321991690179</v>
       </c>
       <c r="H238" t="n">
-        <v>0.1320225853731722</v>
+        <v>0.1269704497455251</v>
       </c>
       <c r="I238" t="n">
-        <v>0.03489310205728124</v>
+        <v>0.06192012908430822</v>
       </c>
       <c r="J238" t="n">
-        <v>0.1320225853731722</v>
+        <v>0.1269704497455251</v>
       </c>
       <c r="K238" t="n">
-        <v>-0.03489310205728124</v>
+        <v>-0.06192012908430822</v>
       </c>
       <c r="L238" t="n">
-        <v>0.00189266049494766</v>
+        <v>0.003003523998178704</v>
       </c>
     </row>
     <row r="239">
@@ -36714,22 +36714,22 @@
         </is>
       </c>
       <c r="G246" t="n">
-        <v>0.1467980017757549</v>
+        <v>0.1413993403704193</v>
       </c>
       <c r="H246" t="n">
-        <v>0.1502322588835416</v>
+        <v>0.1458912537940427</v>
       </c>
       <c r="I246" t="n">
-        <v>-0.01250504235578859</v>
+        <v>-0.06655909640984264</v>
       </c>
       <c r="J246" t="n">
-        <v>0.1502322588835416</v>
+        <v>0.1458912537940427</v>
       </c>
       <c r="K246" t="n">
-        <v>0.01250504235578853</v>
+        <v>0.0665590964098427</v>
       </c>
       <c r="L246" t="n">
-        <v>-0.0009327850347888907</v>
+        <v>-0.002871317444377592</v>
       </c>
     </row>
     <row r="247">
@@ -37108,22 +37108,22 @@
         </is>
       </c>
       <c r="G254" t="n">
-        <v>0.3813725206939891</v>
+        <v>0.3756121520303946</v>
       </c>
       <c r="H254" t="n">
-        <v>0.3843094698150007</v>
+        <v>0.3772464915925169</v>
       </c>
       <c r="I254" t="n">
-        <v>0.2178297700685761</v>
+        <v>0.2718838241226301</v>
       </c>
       <c r="J254" t="n">
-        <v>0.3843094698150007</v>
+        <v>0.3772464915925169</v>
       </c>
       <c r="K254" t="n">
-        <v>-0.2178297700685761</v>
+        <v>-0.2718838241226301</v>
       </c>
       <c r="L254" t="n">
-        <v>-0.009110325892406006</v>
+        <v>-0.006714709681440875</v>
       </c>
     </row>
     <row r="255">
@@ -37504,22 +37504,22 @@
         </is>
       </c>
       <c r="G262" t="n">
-        <v>-0.03367735387772966</v>
+        <v>-0.03173056607759989</v>
       </c>
       <c r="H262" t="n">
-        <v>0.05022947475777662</v>
+        <v>0.04391495247438763</v>
       </c>
       <c r="I262" t="n">
-        <v>-0.05022947475777662</v>
+        <v>-0.04250746703576891</v>
       </c>
       <c r="J262" t="n">
-        <v>-0.04469498367563569</v>
+        <v>-0.04391495247438763</v>
       </c>
       <c r="K262" t="n">
-        <v>0.05022947475777662</v>
+        <v>0.04250746703576891</v>
       </c>
       <c r="L262" t="n">
-        <v>0.1812457974203802</v>
+        <v>0.1783072138176767</v>
       </c>
     </row>
     <row r="263">
@@ -37904,22 +37904,22 @@
         </is>
       </c>
       <c r="G270" t="n">
-        <v>-0.02207868644643315</v>
+        <v>-0.01924952462158368</v>
       </c>
       <c r="H270" t="n">
-        <v>0.03791797188023605</v>
+        <v>0.02744449984184934</v>
       </c>
       <c r="I270" t="n">
-        <v>-0.03791797188023605</v>
+        <v>-0.02462300575508125</v>
       </c>
       <c r="J270" t="n">
-        <v>-0.02830360637105896</v>
+        <v>-0.02744449984184934</v>
       </c>
       <c r="K270" t="n">
-        <v>0.03791797188023605</v>
+        <v>0.02462300575508125</v>
       </c>
       <c r="L270" t="n">
-        <v>0.1461210865561694</v>
+        <v>0.1469271469271469</v>
       </c>
     </row>
     <row r="271">
@@ -38304,22 +38304,22 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>-0.01257960702050918</v>
+        <v>-0.01582425335405882</v>
       </c>
       <c r="H278" t="n">
-        <v>0.02275359055599337</v>
+        <v>0.02431365295848947</v>
       </c>
       <c r="I278" t="n">
-        <v>-0.00533619873242519</v>
+        <v>-0.01691921031543675</v>
       </c>
       <c r="J278" t="n">
-        <v>-0.02275359055599337</v>
+        <v>-0.02431365295848947</v>
       </c>
       <c r="K278" t="n">
-        <v>0.00533619873242519</v>
+        <v>0.01691921031543675</v>
       </c>
       <c r="L278" t="n">
-        <v>0.1421052631578947</v>
+        <v>0.1493975903614458</v>
       </c>
     </row>
     <row r="279">
@@ -38704,22 +38704,22 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>-0.02311527549311079</v>
+        <v>-0.02189523187902753</v>
       </c>
       <c r="H286" t="n">
-        <v>0.07426968747723472</v>
+        <v>0.07126466088730232</v>
       </c>
       <c r="I286" t="n">
-        <v>-0.07426968747723472</v>
+        <v>-0.07126466088730232</v>
       </c>
       <c r="J286" t="n">
-        <v>-0.02702767904530614</v>
+        <v>-0.02624764784405809</v>
       </c>
       <c r="K286" t="n">
-        <v>0.07426968747723472</v>
+        <v>0.07126466088730232</v>
       </c>
       <c r="L286" t="n">
-        <v>0.1386879837584063</v>
+        <v>0.1336571998006976</v>
       </c>
     </row>
     <row r="287">
@@ -39104,22 +39104,22 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>0.2992191154943181</v>
+        <v>0.3167402056954862</v>
       </c>
       <c r="H294" t="n">
-        <v>0.3009808021186827</v>
+        <v>0.32204164455238</v>
       </c>
       <c r="I294" t="n">
         <v>0.2298390034239091</v>
       </c>
       <c r="J294" t="n">
-        <v>0.3009808021186827</v>
+        <v>0.32204164455238</v>
       </c>
       <c r="K294" t="n">
         <v>-0.2298390034239091</v>
       </c>
       <c r="L294" t="n">
-        <v>-0.4599185573007563</v>
+        <v>-0.4744484718306708</v>
       </c>
     </row>
     <row r="295">
@@ -39504,22 +39504,22 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>0.2085510579056185</v>
+        <v>0.2007639067050994</v>
       </c>
       <c r="H302" t="n">
-        <v>0.2911233335761637</v>
+        <v>0.2872623297151599</v>
       </c>
       <c r="I302" t="n">
-        <v>0.2911233335761637</v>
+        <v>0.2872623297151599</v>
       </c>
       <c r="J302" t="n">
-        <v>0.1826103971993931</v>
+        <v>0.1740300539856646</v>
       </c>
       <c r="K302" t="n">
-        <v>-0.2911233335761637</v>
+        <v>-0.2872623297151599</v>
       </c>
       <c r="L302" t="n">
-        <v>-0.2249330361323917</v>
+        <v>-0.2170864859687769</v>
       </c>
     </row>
     <row r="303">
@@ -39904,22 +39904,22 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>0.2063180055234445</v>
+        <v>0.2047867022320149</v>
       </c>
       <c r="H310" t="n">
-        <v>0.3353063305893494</v>
+        <v>0.340023311721425</v>
       </c>
       <c r="I310" t="n">
-        <v>0.3353063305893494</v>
+        <v>0.340023311721425</v>
       </c>
       <c r="J310" t="n">
-        <v>0.1709997265870016</v>
+        <v>0.1683433316714112</v>
       </c>
       <c r="K310" t="n">
-        <v>-0.3353063305893494</v>
+        <v>-0.340023311721425</v>
       </c>
       <c r="L310" t="n">
-        <v>-0.2283853302356455</v>
+        <v>-0.2128444104914693</v>
       </c>
     </row>
     <row r="311">
@@ -40304,22 +40304,22 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>0.3185563587522449</v>
+        <v>0.2887056124835881</v>
       </c>
       <c r="H318" t="n">
-        <v>0.327286081133967</v>
+        <v>0.2914046458765567</v>
       </c>
       <c r="I318" t="n">
         <v>0.2126830334377504</v>
       </c>
       <c r="J318" t="n">
-        <v>0.327286081133967</v>
+        <v>0.2914046458765567</v>
       </c>
       <c r="K318" t="n">
         <v>-0.2126830334377504</v>
       </c>
       <c r="L318" t="n">
-        <v>-0.5527219873150105</v>
+        <v>-0.5263735485698102</v>
       </c>
     </row>
     <row r="319">
@@ -41104,22 +41104,22 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>-0.0506268914829226</v>
+        <v>-0.03951578037181148</v>
       </c>
       <c r="H334" t="n">
-        <v>0.413882863340564</v>
+        <v>0.3117136659436009</v>
       </c>
       <c r="I334" t="n">
-        <v>-0.413882863340564</v>
+        <v>-0.3117136659436009</v>
       </c>
       <c r="J334" t="n">
-        <v>0.0286876584953508</v>
+        <v>0.02826500422654269</v>
       </c>
       <c r="K334" t="n">
-        <v>0.413882863340564</v>
+        <v>0.3117136659436008</v>
       </c>
       <c r="L334" t="n">
-        <v>-0.4939000393545848</v>
+        <v>-0.4018595041322314</v>
       </c>
     </row>
     <row r="335">
@@ -41502,22 +41502,22 @@
         </is>
       </c>
       <c r="G342" t="n">
-        <v>-0.03554219235153087</v>
+        <v>-0.01296623825806706</v>
       </c>
       <c r="H342" t="n">
-        <v>0.4006507592190889</v>
+        <v>0.500650759219089</v>
       </c>
       <c r="I342" t="n">
-        <v>-0.4006507592190889</v>
+        <v>-0.500650759219089</v>
       </c>
       <c r="J342" t="n">
-        <v>0.04801352493660187</v>
+        <v>0.08593617920541</v>
       </c>
       <c r="K342" t="n">
-        <v>0.4006507592190889</v>
+        <v>0.500650759219089</v>
       </c>
       <c r="L342" t="n">
-        <v>-0.4514879739094986</v>
+        <v>-0.5719965427830597</v>
       </c>
     </row>
     <row r="343">
@@ -41902,22 +41902,22 @@
         </is>
       </c>
       <c r="G350" t="n">
-        <v>-0.06321581574499861</v>
+        <v>-0.06356954761624022</v>
       </c>
       <c r="H350" t="n">
-        <v>0.3741865509761388</v>
+        <v>0.2785249457700651</v>
       </c>
       <c r="I350" t="n">
-        <v>-0.3741865509761388</v>
+        <v>-0.2785249457700651</v>
       </c>
       <c r="J350" t="n">
-        <v>0.02608833474218089</v>
+        <v>0.01401098901098901</v>
       </c>
       <c r="K350" t="n">
-        <v>0.3741865509761388</v>
+        <v>0.2785249457700651</v>
       </c>
       <c r="L350" t="n">
-        <v>-0.3122093023255814</v>
+        <v>-0.1896751740139211</v>
       </c>
     </row>
     <row r="351">
@@ -42302,22 +42302,22 @@
         </is>
       </c>
       <c r="G358" t="n">
-        <v>0.3903627716857289</v>
+        <v>0.3792516605746177</v>
       </c>
       <c r="H358" t="n">
-        <v>0.4812235841081994</v>
+        <v>0.4687235841081995</v>
       </c>
       <c r="I358" t="n">
         <v>0.04750542299349247</v>
       </c>
       <c r="J358" t="n">
-        <v>0.4812235841081994</v>
+        <v>0.4687235841081995</v>
       </c>
       <c r="K358" t="n">
         <v>-0.04750542299349247</v>
       </c>
       <c r="L358" t="n">
-        <v>-0.6615417558886509</v>
+        <v>-0.6578682865008959</v>
       </c>
     </row>
     <row r="359">
@@ -42702,22 +42702,22 @@
         </is>
       </c>
       <c r="G366" t="n">
-        <v>0.1555712769720552</v>
+        <v>0.1329953228785913</v>
       </c>
       <c r="H366" t="n">
-        <v>0.3329718004338394</v>
+        <v>0.2351409978308027</v>
       </c>
       <c r="I366" t="n">
-        <v>-0.3329718004338394</v>
+        <v>-0.2351409978308027</v>
       </c>
       <c r="J366" t="n">
-        <v>0.2577451394759087</v>
+        <v>0.2202451394759087</v>
       </c>
       <c r="K366" t="n">
-        <v>0.3329718004338394</v>
+        <v>0.2351409978308027</v>
       </c>
       <c r="L366" t="n">
-        <v>-0.4168274642225439</v>
+        <v>-0.379887793267596</v>
       </c>
     </row>
     <row r="367">
@@ -43100,22 +43100,22 @@
         </is>
       </c>
       <c r="G374" t="n">
-        <v>0.1865739103093189</v>
+        <v>0.1639979562158551</v>
       </c>
       <c r="H374" t="n">
-        <v>0.2687975486052409</v>
+        <v>0.2433748943364328</v>
       </c>
       <c r="I374" t="n">
         <v>-0.1438177874186551</v>
       </c>
       <c r="J374" t="n">
-        <v>0.2687975486052409</v>
+        <v>0.2433748943364328</v>
       </c>
       <c r="K374" t="n">
         <v>0.1438177874186551</v>
       </c>
       <c r="L374" t="n">
-        <v>-0.35860768175583</v>
+        <v>-0.3486661860129776</v>
       </c>
     </row>
     <row r="375">
@@ -43500,22 +43500,22 @@
         </is>
       </c>
       <c r="G382" t="n">
-        <v>0.3738002594033722</v>
+        <v>0.2849113705144833</v>
       </c>
       <c r="H382" t="n">
-        <v>0.4672125950972105</v>
+        <v>0.3672125950972105</v>
       </c>
       <c r="I382" t="n">
         <v>0.02581344902386118</v>
       </c>
       <c r="J382" t="n">
-        <v>0.4672125950972105</v>
+        <v>0.3672125950972105</v>
       </c>
       <c r="K382" t="n">
         <v>-0.02581344902386118</v>
       </c>
       <c r="L382" t="n">
-        <v>-0.706069844789357</v>
+        <v>-0.668569844789357</v>
       </c>
     </row>
     <row r="383">
@@ -43903,19 +43903,19 @@
         <v>-0.191609977324263</v>
       </c>
       <c r="H390" t="n">
-        <v>0.3559907834101383</v>
+        <v>0.2914746543778802</v>
       </c>
       <c r="I390" t="n">
-        <v>-0.3559907834101383</v>
+        <v>-0.2914746543778802</v>
       </c>
       <c r="J390" t="n">
-        <v>-0.1286050948266188</v>
+        <v>-0.1584558410952755</v>
       </c>
       <c r="K390" t="n">
-        <v>0.3559907834101383</v>
+        <v>0.2914746543778802</v>
       </c>
       <c r="L390" t="n">
-        <v>0.03751065643648765</v>
+        <v>0.1551577152600171</v>
       </c>
     </row>
     <row r="391">
@@ -44300,22 +44300,22 @@
         </is>
       </c>
       <c r="G398" t="n">
-        <v>-0.1662887377173091</v>
+        <v>-0.145880574452003</v>
       </c>
       <c r="H398" t="n">
-        <v>0.3565668202764978</v>
+        <v>0.3243087557603687</v>
       </c>
       <c r="I398" t="n">
-        <v>-0.3565668202764978</v>
+        <v>-0.3243087557603687</v>
       </c>
       <c r="J398" t="n">
-        <v>-0.09033778476040848</v>
+        <v>-0.07541241162608012</v>
       </c>
       <c r="K398" t="n">
-        <v>0.3565668202764978</v>
+        <v>0.3243087557603687</v>
       </c>
       <c r="L398" t="n">
-        <v>0.1589147286821706</v>
+        <v>0.07558139534883723</v>
       </c>
     </row>
     <row r="399">
@@ -44700,7 +44700,7 @@
         </is>
       </c>
       <c r="G406" t="n">
-        <v>-0.1405895691609977</v>
+        <v>-0.1352985638699924</v>
       </c>
       <c r="H406" t="n">
         <v>0.3421658986175115</v>
@@ -44709,13 +44709,13 @@
         <v>-0.3421658986175115</v>
       </c>
       <c r="J406" t="n">
-        <v>-0.06037481764111771</v>
+        <v>-0.05285602064863651</v>
       </c>
       <c r="K406" t="n">
         <v>0.3421658986175115</v>
       </c>
       <c r="L406" t="n">
-        <v>0.0357142857142857</v>
+        <v>0.01829268292682928</v>
       </c>
     </row>
     <row r="407">
@@ -45100,7 +45100,7 @@
         </is>
       </c>
       <c r="G414" t="n">
-        <v>-0.163265306122449</v>
+        <v>-0.1315192743764172</v>
       </c>
       <c r="H414" t="n">
         <v>0.2632488479262673</v>
@@ -45109,13 +45109,13 @@
         <v>-0.2632488479262673</v>
       </c>
       <c r="J414" t="n">
-        <v>-0.1281562114240826</v>
+        <v>-0.08304342946919538</v>
       </c>
       <c r="K414" t="n">
         <v>0.2632488479262673</v>
       </c>
       <c r="L414" t="n">
-        <v>0.1759259259259259</v>
+        <v>0.1041666666666666</v>
       </c>
     </row>
     <row r="415">
@@ -45500,22 +45500,22 @@
         </is>
       </c>
       <c r="G422" t="n">
-        <v>0.1281179138321996</v>
+        <v>0.1485260770975056</v>
       </c>
       <c r="H422" t="n">
-        <v>0.1339916956570531</v>
+        <v>0.1489170687913814</v>
       </c>
       <c r="I422" t="n">
-        <v>0.09792626728110598</v>
+        <v>0.130184331797235</v>
       </c>
       <c r="J422" t="n">
-        <v>0.1339916956570531</v>
+        <v>0.1489170687913814</v>
       </c>
       <c r="K422" t="n">
-        <v>-0.09792626728110609</v>
+        <v>-0.1301843317972351</v>
       </c>
       <c r="L422" t="n">
-        <v>-0.23</v>
+        <v>-0.2314814814814815</v>
       </c>
     </row>
     <row r="423">
@@ -45900,22 +45900,22 @@
         </is>
       </c>
       <c r="G430" t="n">
-        <v>0.05857898715041571</v>
+        <v>0.05328798185941042</v>
       </c>
       <c r="H430" t="n">
-        <v>0.08147233756031871</v>
+        <v>0.07395354056783751</v>
       </c>
       <c r="I430" t="n">
         <v>-0.0195852534562212</v>
       </c>
       <c r="J430" t="n">
-        <v>0.08147233756031871</v>
+        <v>0.07395354056783751</v>
       </c>
       <c r="K430" t="n">
         <v>0.0195852534562212</v>
       </c>
       <c r="L430" t="n">
-        <v>-0.1391147244805782</v>
+        <v>-0.1216931216931217</v>
       </c>
     </row>
     <row r="431">
@@ -46300,22 +46300,22 @@
         </is>
       </c>
       <c r="G438" t="n">
-        <v>0.03590325018896451</v>
+        <v>0.02569916855631144</v>
       </c>
       <c r="H438" t="n">
         <v>0.02872853776231624</v>
       </c>
       <c r="I438" t="n">
-        <v>0.02361751152073732</v>
+        <v>-0.008640552995391682</v>
       </c>
       <c r="J438" t="n">
         <v>0.02872853776231624</v>
       </c>
       <c r="K438" t="n">
-        <v>-0.02361751152073732</v>
+        <v>0.008640552995391682</v>
       </c>
       <c r="L438" t="n">
-        <v>-0.009738283627510613</v>
+        <v>-0.02264150943396226</v>
       </c>
     </row>
     <row r="439">
@@ -46700,22 +46700,22 @@
         </is>
       </c>
       <c r="G446" t="n">
-        <v>0.13567649281935</v>
+        <v>0.1764928193499622</v>
       </c>
       <c r="H446" t="n">
-        <v>0.1411738300976322</v>
+        <v>0.1859499495006172</v>
       </c>
       <c r="I446" t="n">
-        <v>0.09850230414746547</v>
+        <v>0.1307603686635945</v>
       </c>
       <c r="J446" t="n">
-        <v>0.1411738300976322</v>
+        <v>0.1859499495006172</v>
       </c>
       <c r="K446" t="n">
-        <v>-0.09850230414746541</v>
+        <v>-0.1307603686635944</v>
       </c>
       <c r="L446" t="n">
-        <v>-0.1650717703349283</v>
+        <v>-0.1970128022759602</v>
       </c>
     </row>
     <row r="447">
@@ -47100,22 +47100,22 @@
         </is>
       </c>
       <c r="G454" t="n">
-        <v>-0.09776453055141579</v>
+        <v>-0.07352210630899156</v>
       </c>
       <c r="H454" t="n">
-        <v>0.1761904761904762</v>
+        <v>0.2</v>
       </c>
       <c r="I454" t="n">
-        <v>-0.1761904761904762</v>
+        <v>-0.2</v>
       </c>
       <c r="J454" t="n">
-        <v>-0.1286031042128603</v>
+        <v>-0.08795269770879527</v>
       </c>
       <c r="K454" t="n">
-        <v>0.1761904761904762</v>
+        <v>0.2</v>
       </c>
       <c r="L454" t="n">
-        <v>0.25</v>
+        <v>0.1899999999999999</v>
       </c>
     </row>
     <row r="455">
@@ -47900,22 +47900,22 @@
         </is>
       </c>
       <c r="G470" t="n">
-        <v>-0.1708395429706905</v>
+        <v>-0.1526577247888724</v>
       </c>
       <c r="H470" t="n">
-        <v>0.3412698412698413</v>
+        <v>0.2698412698412699</v>
       </c>
       <c r="I470" t="n">
-        <v>-0.3412698412698413</v>
+        <v>-0.2698412698412699</v>
       </c>
       <c r="J470" t="n">
         <v>-0.1708372927885123</v>
       </c>
       <c r="K470" t="n">
-        <v>0.3412698412698413</v>
+        <v>0.2698412698412699</v>
       </c>
       <c r="L470" t="n">
-        <v>0.267741935483871</v>
+        <v>0.2915254237288136</v>
       </c>
     </row>
     <row r="471">
@@ -48300,7 +48300,7 @@
         </is>
       </c>
       <c r="G478" t="n">
-        <v>-0.06527570789865872</v>
+        <v>-0.05101838052657724</v>
       </c>
       <c r="H478" t="n">
         <v>0.2063492063492063</v>
@@ -48309,13 +48309,13 @@
         <v>-0.2063492063492063</v>
       </c>
       <c r="J478" t="n">
-        <v>-0.04719670573329109</v>
+        <v>-0.02607961144546511</v>
       </c>
       <c r="K478" t="n">
         <v>0.2063492063492064</v>
       </c>
       <c r="L478" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.07692307692307698</v>
       </c>
     </row>
     <row r="479">
@@ -48700,19 +48700,19 @@
         </is>
       </c>
       <c r="G486" t="n">
-        <v>0.1899155489319423</v>
+        <v>0.2472925981122702</v>
       </c>
       <c r="H486" t="n">
-        <v>0.1825396825396825</v>
+        <v>0.2714285714285714</v>
       </c>
       <c r="I486" t="n">
-        <v>0.1825396825396825</v>
+        <v>0.2714285714285714</v>
       </c>
       <c r="J486" t="n">
-        <v>0.1541547883011298</v>
+        <v>0.1931158272621687</v>
       </c>
       <c r="K486" t="n">
-        <v>-0.1825396825396826</v>
+        <v>-0.2714285714285715</v>
       </c>
       <c r="L486" t="n">
         <v>-0.1160714285714286</v>
@@ -49100,22 +49100,22 @@
         </is>
       </c>
       <c r="G494" t="n">
-        <v>0.1991554893194238</v>
+        <v>0.1767014406358669</v>
       </c>
       <c r="H494" t="n">
-        <v>0.1832963784183296</v>
+        <v>0.1443353394572907</v>
       </c>
       <c r="I494" t="n">
-        <v>0.1285714285714286</v>
+        <v>0.126984126984127</v>
       </c>
       <c r="J494" t="n">
-        <v>0.1832963784183296</v>
+        <v>0.1443353394572907</v>
       </c>
       <c r="K494" t="n">
-        <v>-0.1285714285714286</v>
+        <v>-0.126984126984127</v>
       </c>
       <c r="L494" t="n">
-        <v>-0.07380952380952377</v>
+        <v>-0.03929430633520448</v>
       </c>
     </row>
     <row r="495">
@@ -49500,22 +49500,22 @@
         </is>
       </c>
       <c r="G502" t="n">
-        <v>0.2208643815201192</v>
+        <v>0.1820168902136115</v>
       </c>
       <c r="H502" t="n">
-        <v>0.1994509555485165</v>
+        <v>0.1653468482736775</v>
       </c>
       <c r="I502" t="n">
-        <v>0.1158730158730159</v>
+        <v>0.0714285714285714</v>
       </c>
       <c r="J502" t="n">
-        <v>0.1994509555485165</v>
+        <v>0.1653468482736775</v>
       </c>
       <c r="K502" t="n">
-        <v>-0.1158730158730159</v>
+        <v>-0.0714285714285714</v>
       </c>
       <c r="L502" t="n">
-        <v>-0.04351395730706076</v>
+        <v>-0.02583979328165376</v>
       </c>
     </row>
     <row r="503">
@@ -49900,22 +49900,22 @@
         </is>
       </c>
       <c r="G510" t="n">
-        <v>0.1574764033780427</v>
+        <v>0.1410829607550919</v>
       </c>
       <c r="H510" t="n">
-        <v>0.1349206349206349</v>
+        <v>0.1126984126984127</v>
       </c>
       <c r="I510" t="n">
-        <v>0.1349206349206349</v>
+        <v>0.1126984126984127</v>
       </c>
       <c r="J510" t="n">
-        <v>0.1249076127124908</v>
+        <v>0.1119205997254778</v>
       </c>
       <c r="K510" t="n">
-        <v>-0.1349206349206349</v>
+        <v>-0.1126984126984127</v>
       </c>
       <c r="L510" t="n">
-        <v>-0.06176470588235294</v>
+        <v>-0.05625000000000002</v>
       </c>
     </row>
     <row r="511">

</xml_diff>